<commit_message>
chore: finalize delivery package and member test coverage
</commit_message>
<xml_diff>
--- a/Docs/deliverables/product-backlog/product-backlog-group14.xlsx
+++ b/Docs/deliverables/product-backlog/product-backlog-group14.xlsx
@@ -7,7 +7,7 @@
     <workbookView windowWidth="25600" windowHeight="10480"/>
   </bookViews>
   <sheets>
-    <sheet name="产品待办列表" sheetId="1" r:id="rId1"/>
+    <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,370 +29,370 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="106">
   <si>
-    <t>用户故事编号</t>
-  </si>
-  <si>
-    <t>用户故事名称</t>
-  </si>
-  <si>
-    <t>描述</t>
-  </si>
-  <si>
-    <t>优先级</t>
-  </si>
-  <si>
-    <t>迭代编号</t>
-  </si>
-  <si>
-    <t>验收标准</t>
-  </si>
-  <si>
-    <t>估算</t>
-  </si>
-  <si>
-    <t>备注</t>
-  </si>
-  <si>
-    <t>开始日期（或计划日期）</t>
-  </si>
-  <si>
-    <t>完成日期（或计划日期）</t>
+    <t>User Story ID</t>
+  </si>
+  <si>
+    <t>User Story Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Iteration</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Estimate</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Start Date (or Planned Date)</t>
+  </si>
+  <si>
+    <t>Completion Date (or Planned Date)</t>
   </si>
   <si>
     <t>US001</t>
   </si>
   <si>
-    <t>用户注册</t>
-  </si>
-  <si>
-    <t>作为新用户，我希望注册账号，以便访问系统</t>
-  </si>
-  <si>
-    <t>高</t>
-  </si>
-  <si>
-    <t>1. 用户可以输入姓名、邮箱和密码
-2. 系统校验邮箱格式
-3. 系统检查密码强度
-4. 账号成功创建</t>
-  </si>
-  <si>
-    <t>第二阶段 - 第 1 次迭代</t>
+    <t>User Registration</t>
+  </si>
+  <si>
+    <t>As a new user, I want to register an account so that I can access the system.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>1. The user can enter name, email, and password
+2. The system validates the email format
+3. The system checks password strength
+4. The account is created successfully</t>
+  </si>
+  <si>
+    <t>Phase 2 - Iteration 1</t>
   </si>
   <si>
     <t>US002</t>
   </si>
   <si>
-    <t>用户登录</t>
-  </si>
-  <si>
-    <t>作为已注册用户，我希望登录系统，以便访问我的个性化仪表盘</t>
-  </si>
-  <si>
-    <t>1. 用户可以输入邮箱和密码
-2. 凭据无效时显示错误信息
-3. 登录成功后创建会话</t>
+    <t>User Login</t>
+  </si>
+  <si>
+    <t>As a registered user, I want to log in so that I can access my personalized dashboard.</t>
+  </si>
+  <si>
+    <t>1. The user can enter email and password
+2. An error message is shown for invalid credentials
+3. A session is created after successful login</t>
   </si>
   <si>
     <t>US003</t>
   </si>
   <si>
-    <t>角色选择</t>
-  </si>
-  <si>
-    <t>作为用户，我希望选择自己的角色（TA 或 MO），以便访问对应功能</t>
-  </si>
-  <si>
-    <t>1. 用户可以选择 TA 或 MO 角色
-2. 角色保存到用户资料中
-3. 界面根据所选角色调整</t>
+    <t>Role Selection</t>
+  </si>
+  <si>
+    <t>As a user, I want to choose my role (TA or MO) so that I can access the corresponding features.</t>
+  </si>
+  <si>
+    <t>1. The user can choose the TA or MO role
+2. The role is saved in the user profile
+3. The interface adapts to the selected role</t>
   </si>
   <si>
     <t>US004</t>
   </si>
   <si>
-    <t>TA 个人资料创建</t>
-  </si>
-  <si>
-    <t>作为 TA 申请人，我希望创建个人资料，以便 MO 审核我的信息</t>
-  </si>
-  <si>
-    <t>1. TA 可以输入个人信息（姓名、学号、专业、年级）
-2. TA 可以添加联系方式
-3. 个人资料保存到系统中</t>
+    <t>TA Profile Creation</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to create a profile so that the MO can review my information.</t>
+  </si>
+  <si>
+    <t>1. The TA can enter personal information (name, student ID, major, year)
+2. The TA can add contact details
+3. The profile is saved in the system</t>
   </si>
   <si>
     <t>US005</t>
   </si>
   <si>
-    <t>简历上传</t>
-  </si>
-  <si>
-    <t>作为 TA 申请人，我希望上传简历，以便 MO 审核我的资质</t>
-  </si>
-  <si>
-    <t>1. TA 可以上传 PDF/DOC 格式简历
-2. 系统限制文件大小（最大 5MB）
-3. 简历被保存并关联到个人资料</t>
+    <t>Resume Upload</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to upload my resume so that the MO can review my qualifications.</t>
+  </si>
+  <si>
+    <t>1. The TA can upload a PDF/DOC resume
+2. The system limits file size (maximum 5 MB)
+3. The resume is saved and linked to the profile</t>
   </si>
   <si>
     <t>US006</t>
   </si>
   <si>
-    <t>技能声明</t>
-  </si>
-  <si>
-    <t>作为 TA 申请人，我希望声明自己的技能，以便系统为我匹配合适岗位</t>
-  </si>
-  <si>
-    <t>中</t>
-  </si>
-  <si>
-    <t>1. TA 可以从预定义列表中选择技能
-2. TA 可以添加自定义技能
-3. 技能保存到个人资料中</t>
+    <t>Skill Declaration</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to declare my skills so that the system can match me with suitable positions.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>1. The TA can select skills from a predefined list
+2. The TA can add custom skills
+3. Skills are saved in the profile</t>
   </si>
   <si>
     <t>US007</t>
   </si>
   <si>
-    <t>岗位发布创建</t>
-  </si>
-  <si>
-    <t>作为 MO，我希望创建并发布岗位，以便 TA 查看并申请</t>
-  </si>
-  <si>
-    <t>1. MO 可以输入岗位标题和描述
-2. MO 可以指定所需技能
-3. MO 可以设置截止日期
-4. 岗位发布后对 TA 可见</t>
-  </si>
-  <si>
-    <t>第二阶段 - 第 2 次迭代</t>
+    <t>Job Posting Creation</t>
+  </si>
+  <si>
+    <t>As an MO, I want to create and publish positions so that TAs can view and apply for them.</t>
+  </si>
+  <si>
+    <t>1. The MO can enter the job title and description
+2. The MO can specify required skills
+3. The MO can set an application deadline
+4. The posting is visible to TAs after publication</t>
+  </si>
+  <si>
+    <t>Phase 2 - Iteration 2</t>
   </si>
   <si>
     <t>US008</t>
   </si>
   <si>
-    <t>岗位列表展示</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望查看可申请岗位，以便找到合适职位</t>
-  </si>
-  <si>
-    <t>1. 显示所有有效岗位
-2. 岗位按截止日期排序
-3. 点击后可查看岗位详情</t>
+    <t>Job List Display</t>
+  </si>
+  <si>
+    <t>As a TA, I want to view available positions so that I can find a suitable role.</t>
+  </si>
+  <si>
+    <t>1. All active positions are displayed
+2. Positions are sorted by deadline
+3. Clicking a position opens its details</t>
   </si>
   <si>
     <t>US009</t>
   </si>
   <si>
-    <t>岗位搜索 / 筛选</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望搜索和筛选岗位，以便找到与技能匹配的职位</t>
-  </si>
-  <si>
-    <t>1. TA 可以按关键词搜索
-2. TA 可以按所需技能筛选
-3. 筛选结果实时更新</t>
+    <t>Job Search / Filtering</t>
+  </si>
+  <si>
+    <t>As a TA, I want to search and filter positions so that I can find roles matching my skills.</t>
+  </si>
+  <si>
+    <t>1. The TA can search by keyword
+2. The TA can filter by required skills
+3. Filtered results update in real time</t>
   </si>
   <si>
     <t>US010</t>
   </si>
   <si>
-    <t>岗位申请</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望申请岗位，以便获得该职位的考虑机会</t>
-  </si>
-  <si>
-    <t>1. TA 可以在申请前查看岗位详情
-2. TA 可以提交申请
-3. 申请关联到 TA 个人资料
-4. 提交后显示确认信息</t>
+    <t>Job Application</t>
+  </si>
+  <si>
+    <t>As a TA, I want to apply for a position so that I can be considered for that role.</t>
+  </si>
+  <si>
+    <t>1. The TA can review job details before applying
+2. The TA can submit an application
+3. The application is linked to the TA profile
+4. A confirmation message is shown after submission</t>
   </si>
   <si>
     <t>US011</t>
   </si>
   <si>
-    <t>申请状态查看</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望查看申请状态，以便跟踪我的岗位申请</t>
-  </si>
-  <si>
-    <t>1. TA 可以查看自己的全部申请
-2. 显示状态（待审核 / 已接受 / 已拒绝）
-3. 状态实时更新</t>
+    <t>Application Status View</t>
+  </si>
+  <si>
+    <t>As a TA, I want to view application status so that I can track my job applications.</t>
+  </si>
+  <si>
+    <t>1. The TA can view all of their applications
+2. Status is displayed (pending / accepted / rejected)
+3. Status updates in real time</t>
   </si>
   <si>
     <t>US012</t>
   </si>
   <si>
-    <t>申请人列表查看</t>
-  </si>
-  <si>
-    <t>作为 MO，我希望查看岗位的所有申请人，以便进行评估</t>
-  </si>
-  <si>
-    <t>1. MO 可以查看申请人列表
-2. MO 可以查看申请人资料
-3. MO 可以查看简历</t>
+    <t>Applicant List View</t>
+  </si>
+  <si>
+    <t>As an MO, I want to view all applicants for a position so that I can evaluate them.</t>
+  </si>
+  <si>
+    <t>1. The MO can view the applicant list
+2. The MO can view applicant profiles
+3. The MO can view resumes</t>
   </si>
   <si>
     <t>US013</t>
   </si>
   <si>
-    <t>申请人选择</t>
-  </si>
-  <si>
-    <t>作为 MO，我希望选择申请人，以便向其提供 TA 岗位</t>
-  </si>
-  <si>
-    <t>1. MO 可以接受或拒绝申请人
-2. TA 会收到决定通知
-3. 申请状态被更新</t>
+    <t>Applicant Selection</t>
+  </si>
+  <si>
+    <t>As an MO, I want to select applicants so that I can offer them TA positions.</t>
+  </si>
+  <si>
+    <t>1. The MO can accept or reject applicants
+2. The TA receives a decision notification
+3. The application status is updated</t>
   </si>
   <si>
     <t>US014</t>
   </si>
   <si>
-    <t>退出登录</t>
-  </si>
-  <si>
-    <t>作为用户，我希望退出登录，以便安全离开系统</t>
-  </si>
-  <si>
-    <t>1. 用户可以点击退出登录
-2. 会话被终止
-3. 系统重定向到登录页面</t>
+    <t>Logout</t>
+  </si>
+  <si>
+    <t>As a user, I want to log out so that I can leave the system safely.</t>
+  </si>
+  <si>
+    <t>1. The user can click logout
+2. The session is terminated
+3. The system redirects to the login page</t>
   </si>
   <si>
     <t>US015</t>
   </si>
   <si>
-    <t>个人资料编辑</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望编辑个人资料，以便保持信息最新</t>
-  </si>
-  <si>
-    <t>1. TA 可以修改个人资料详情
-2. 修改会立即保存
-3. 简历可以更新</t>
-  </si>
-  <si>
-    <t>第二阶段 - 第 3 次迭代</t>
+    <t>Profile Editing</t>
+  </si>
+  <si>
+    <t>As a TA, I want to edit my profile so that my information stays up to date.</t>
+  </si>
+  <si>
+    <t>1. The TA can modify profile details
+2. Changes are saved immediately
+3. The resume can be updated</t>
+  </si>
+  <si>
+    <t>Phase 2 - Iteration 3</t>
   </si>
   <si>
     <t>US016</t>
   </si>
   <si>
-    <t>AI 技能匹配</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望获得 AI 驱动的岗位推荐，以便找到最匹配的职位</t>
-  </si>
-  <si>
-    <t>1. 系统分析 TA 技能和岗位要求
-2. 每个岗位显示匹配百分比
-3. 显示前 5 个推荐岗位</t>
-  </si>
-  <si>
-    <t>第三阶段 - 第 3 次迭代</t>
+    <t>AI Skill Matching</t>
+  </si>
+  <si>
+    <t>As a TA, I want to receive AI-driven job recommendations so that I can find the best-matching positions.</t>
+  </si>
+  <si>
+    <t>1. The system analyzes TA skills and job requirements
+2. Each job displays a match percentage
+3. The top 5 recommended positions are displayed</t>
+  </si>
+  <si>
+    <t>Phase 3 - Iteration 3</t>
   </si>
   <si>
     <t>US017</t>
   </si>
   <si>
-    <t>AI 缺失技能检测</t>
-  </si>
-  <si>
-    <t>作为 TA，我希望了解自己针对某岗位缺少哪些技能，以便提升资质</t>
-  </si>
-  <si>
-    <t>1. 系统识别缺失的必需技能
-2. 提供技能提升建议
-3. 推荐学习资源</t>
+    <t>AI Missing-Skill Detection</t>
+  </si>
+  <si>
+    <t>As a TA, I want to understand which skills I am missing for a position so that I can improve my qualifications.</t>
+  </si>
+  <si>
+    <t>1. The system identifies missing required skills
+2. Skill-improvement suggestions are provided
+3. Learning resources are recommended</t>
   </si>
   <si>
     <t>US018</t>
   </si>
   <si>
-    <t>管理员工作量统计</t>
-  </si>
-  <si>
-    <t>作为管理员，我希望查看工作量统计，以便监控系统使用情况</t>
-  </si>
-  <si>
-    <t>低</t>
-  </si>
-  <si>
-    <t>1. 显示活跃 TA 数量
-2. 显示岗位发布数量
-3. 可查看申请统计
-4. 数据可导出</t>
+    <t>Admin Workload Statistics</t>
+  </si>
+  <si>
+    <t>As an admin, I want to view workload statistics so that I can monitor system usage.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>1. The number of active TAs is displayed
+2. The number of job postings is displayed
+3. Application statistics can be viewed
+4. Data can be exported</t>
   </si>
   <si>
     <t>US019</t>
   </si>
   <si>
-    <t>岗位发布管理</t>
-  </si>
-  <si>
-    <t>作为 MO，我希望管理自己发布的岗位，以便更新或移除它们</t>
-  </si>
-  <si>
-    <t>1. MO 可以编辑岗位详情
-2. MO 可以关闭 / 删除岗位发布
-3. 受影响的申请人会收到通知</t>
-  </si>
-  <si>
-    <t>第三阶段 - 第 4 次迭代</t>
+    <t>Job Posting Management</t>
+  </si>
+  <si>
+    <t>As an MO, I want to manage my own postings so that I can update or remove them.</t>
+  </si>
+  <si>
+    <t>1. The MO can edit job details
+2. The MO can close/delete job postings
+3. Affected applicants receive notifications</t>
+  </si>
+  <si>
+    <t>Phase 3 - Iteration 4</t>
   </si>
   <si>
     <t>US020</t>
   </si>
   <si>
-    <t>邮件通知</t>
-  </si>
-  <si>
-    <t>作为用户，我希望接收邮件通知，以便及时了解重要更新</t>
-  </si>
-  <si>
-    <t>1. 申请状态变化会触发邮件
-2. 新岗位发布会通知匹配的 TA
-3. 系统发送截止日期提醒</t>
+    <t>Email Notifications</t>
+  </si>
+  <si>
+    <t>As a user, I want to receive email notifications so that I can learn about important updates promptly.</t>
+  </si>
+  <si>
+    <t>1. Application status changes trigger emails
+2. New postings notify matching TAs
+3. The system sends deadline reminders</t>
   </si>
   <si>
     <t>US021</t>
   </si>
   <si>
-    <t>性能优化</t>
-  </si>
-  <si>
-    <t>作为系统管理员，我希望系统保持最佳性能，以便用户获得流畅体验</t>
-  </si>
-  <si>
-    <t>1. 页面加载时间小于 2 秒
-2. 数据库查询已优化
-3. 已实现缓存机制</t>
+    <t>Performance Optimization</t>
+  </si>
+  <si>
+    <t>As a system admin, I want the system to maintain optimal performance so that users have a smooth experience.</t>
+  </si>
+  <si>
+    <t>1. Page load time is under 2 seconds
+2. Database queries are optimized
+3. A caching mechanism is implemented</t>
   </si>
   <si>
     <t>US022</t>
   </si>
   <si>
-    <t>用户手册</t>
-  </si>
-  <si>
-    <t>作为用户，我希望访问用户手册，以便学习如何使用系统</t>
-  </si>
-  <si>
-    <t>1. 系统中提供用户手册
-2. 每个功能都有帮助章节
-3. 文档可搜索</t>
+    <t>User Manual</t>
+  </si>
+  <si>
+    <t>As a user, I want to access the user manual so that I can learn how to use the system.</t>
+  </si>
+  <si>
+    <t>1. A user manual is provided in the system
+2. Each feature has a help section
+3. The documentation is searchable</t>
   </si>
 </sst>
 </file>
@@ -409,7 +409,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -417,7 +417,7 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -425,14 +425,14 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -440,7 +440,7 @@
       <b/>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -448,7 +448,7 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -456,7 +456,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -464,7 +464,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -472,14 +472,14 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -487,7 +487,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -495,7 +495,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -503,14 +503,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -518,42 +518,42 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -1056,55 +1056,55 @@
     </xf>
   </cellXfs>
   <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent 1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent 2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent 3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent 4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent 5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
@@ -1163,8 +1163,8 @@
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Hans" typeface="Arial"/>
+        <a:font script="Hant" typeface="Arial"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1198,8 +1198,8 @@
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Hans" typeface="Arial"/>
+        <a:font script="Hant" typeface="Arial"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>

</xml_diff>